<commit_message>
REALIZANDO EJERCICIOS DE NIVEL AVANZADO DE EXCEL
</commit_message>
<xml_diff>
--- a/Nivel Avanzado/Examen Nivel Avanzado.xlsx
+++ b/Nivel Avanzado/Examen Nivel Avanzado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\db\Nik Denilson\Cursos\EXCEL\Nivel Avanzado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84214E7D-8F9E-4361-A5ED-3E4620D2CEAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D303568E-39D2-47E5-8966-7C2F152EBB2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -816,7 +816,7 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -855,278 +855,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="81">
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
+  <dxfs count="25">
     <dxf>
       <font>
         <b/>
@@ -10723,14 +10458,14 @@
     <dataField name="Suma de Venta" fld="8" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="70">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
@@ -10829,7 +10564,7 @@
     <dataField name="Suma de Venta" fld="8" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="71">
+    <format dxfId="15">
       <pivotArea dataOnly="0" fieldPosition="0">
         <references count="1">
           <reference field="4" count="0"/>
@@ -10923,10 +10658,10 @@
     <dataField name="Recuento" fld="8" subtotal="count" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="57">
+    <format dxfId="1">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -11023,10 +10758,10 @@
     <dataField name="Cantidad Empleados" fld="0" subtotal="count" baseField="7" baseItem="1"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="59">
+    <format dxfId="3">
       <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -11209,10 +10944,10 @@
     <dataField name="Salario Anual" fld="4" baseField="3" baseItem="0" numFmtId="167"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="62">
+    <format dxfId="6">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -11222,7 +10957,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="4">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -11350,21 +11085,21 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC378051-9E72-4BB2-9AB0-F6E23C44A7CC}" name="ventas" displayName="ventas" ref="B18:J68" totalsRowShown="0">
   <autoFilter ref="B18:J68" xr:uid="{FC378051-9E72-4BB2-9AB0-F6E23C44A7CC}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D476CF5C-0E1B-40EE-A62B-72E29404A39A}" name="Sale ID" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{CAEA63EE-5517-4029-80DE-DE7ABE2E5FE3}" name="Fecha_Venta" dataDxfId="79"/>
-    <tableColumn id="9" xr3:uid="{2C9B66F8-7131-4DF0-9EB5-8DA6CE795516}" name="AÑO" dataDxfId="78">
+    <tableColumn id="1" xr3:uid="{D476CF5C-0E1B-40EE-A62B-72E29404A39A}" name="Sale ID" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{CAEA63EE-5517-4029-80DE-DE7ABE2E5FE3}" name="Fecha_Venta" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{2C9B66F8-7131-4DF0-9EB5-8DA6CE795516}" name="AÑO" dataDxfId="22">
       <calculatedColumnFormula>YEAR(ventas[[#This Row],[Fecha_Venta]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{5CF4337F-83E1-4D83-A9C4-E333AA16FA95}" name="MES" dataDxfId="77">
+    <tableColumn id="10" xr3:uid="{5CF4337F-83E1-4D83-A9C4-E333AA16FA95}" name="MES" dataDxfId="21">
       <calculatedColumnFormula>MONTH(ventas[[#This Row],[Fecha_Venta]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{72DA8C50-CDA6-43E5-9431-CA09B2A1FCBE}" name="Categoria" dataDxfId="76"/>
-    <tableColumn id="4" xr3:uid="{F2936085-E31D-4D2E-AEFB-560F58DED709}" name="Nombre Producto" dataDxfId="75"/>
-    <tableColumn id="5" xr3:uid="{52293038-8FA6-493E-80D2-45B3340AF0BE}" name="Unidades Vendidas" dataDxfId="74"/>
-    <tableColumn id="7" xr3:uid="{6EAB6895-F3DA-4781-8FF6-2EA5365F5DE0}" name="Precio" dataDxfId="73" dataCellStyle="Millares">
+    <tableColumn id="3" xr3:uid="{72DA8C50-CDA6-43E5-9431-CA09B2A1FCBE}" name="Categoria" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{F2936085-E31D-4D2E-AEFB-560F58DED709}" name="Nombre Producto" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{52293038-8FA6-493E-80D2-45B3340AF0BE}" name="Unidades Vendidas" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{6EAB6895-F3DA-4781-8FF6-2EA5365F5DE0}" name="Precio" dataDxfId="17" dataCellStyle="Millares">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ventas[[#This Row],[Nombre Producto]],precios[Nombre Producto],precios[Price (USD)],"-",0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{CD38CA07-791D-439F-AC3E-94E715454305}" name="Venta" dataDxfId="72">
+    <tableColumn id="8" xr3:uid="{CD38CA07-791D-439F-AC3E-94E715454305}" name="Venta" dataDxfId="16">
       <calculatedColumnFormula>PRODUCT(ventas[[#This Row],[Unidades Vendidas]:[Precio]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11385,7 +11120,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8E1BDC09-0A31-468E-854C-B0887DE35573}" name="RH" displayName="RH" ref="A23:I73" totalsRowShown="0" headerRowDxfId="68" headerRowBorderDxfId="67" tableBorderDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8E1BDC09-0A31-468E-854C-B0887DE35573}" name="RH" displayName="RH" ref="A23:I73" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10">
   <autoFilter ref="A23:I73" xr:uid="{8E1BDC09-0A31-468E-854C-B0887DE35573}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{CA5BADCE-87A3-4C6C-8C9E-32804204CFD6}" name="Nombre"/>
@@ -11393,9 +11128,9 @@
     <tableColumn id="3" xr3:uid="{5A6F001D-C24B-403D-8DFA-ED4932F47AF0}" name="Apellido Materno"/>
     <tableColumn id="4" xr3:uid="{4C5A6D7B-ADA5-4DAD-8FCE-5614D22DCB1A}" name="Puesto"/>
     <tableColumn id="5" xr3:uid="{F917D2AA-F2F7-4449-8B16-DDBE5DBD687A}" name="Salario Anual (USD)"/>
-    <tableColumn id="6" xr3:uid="{5150356B-0BC9-4651-9491-E2CA4FBB946A}" name="Fecha Contratación" dataDxfId="65"/>
-    <tableColumn id="7" xr3:uid="{479B983A-A0DC-4CB3-83F9-1DA14406634A}" name="Fecha Nacimiento" dataDxfId="64"/>
-    <tableColumn id="9" xr3:uid="{40E590F7-C3A8-4023-B335-4C8D470BAB64}" name="EdadTrabajador" dataDxfId="63">
+    <tableColumn id="6" xr3:uid="{5150356B-0BC9-4651-9491-E2CA4FBB946A}" name="Fecha Contratación" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{479B983A-A0DC-4CB3-83F9-1DA14406634A}" name="Fecha Nacimiento" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{40E590F7-C3A8-4023-B335-4C8D470BAB64}" name="EdadTrabajador" dataDxfId="7">
       <calculatedColumnFormula>INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{B2B75107-054A-4454-B3A1-24B9FCDE6668}" name="Género"/>
@@ -14177,7 +13912,7 @@
       </c>
       <c r="H24" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I24" t="s">
         <v>13</v>
@@ -14357,7 +14092,7 @@
       </c>
       <c r="H30" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I30" t="s">
         <v>13</v>
@@ -14447,7 +14182,7 @@
       </c>
       <c r="H33" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I33" t="s">
         <v>22</v>
@@ -14477,7 +14212,7 @@
       </c>
       <c r="H34" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I34" t="s">
         <v>22</v>
@@ -14807,7 +14542,7 @@
       </c>
       <c r="H45" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I45" t="s">
         <v>22</v>
@@ -14897,7 +14632,7 @@
       </c>
       <c r="H48" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I48" t="s">
         <v>13</v>
@@ -15670,7 +15405,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A6:D41"/>
+  <dimension ref="A6:D93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
@@ -15693,7 +15428,7 @@
       <c r="B7" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7">
         <v>11</v>
       </c>
       <c r="D7" s="18">
@@ -15704,7 +15439,7 @@
       <c r="B8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8">
         <v>9</v>
       </c>
       <c r="D8" s="18">
@@ -15715,7 +15450,7 @@
       <c r="B9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9">
         <v>7</v>
       </c>
       <c r="D9" s="18">
@@ -15726,7 +15461,7 @@
       <c r="B10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10">
         <v>7</v>
       </c>
       <c r="D10" s="18">
@@ -15737,7 +15472,7 @@
       <c r="B11" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11">
         <v>6</v>
       </c>
       <c r="D11" s="18">
@@ -15748,7 +15483,7 @@
       <c r="B12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12">
         <v>5</v>
       </c>
       <c r="D12" s="18">
@@ -15759,7 +15494,7 @@
       <c r="B13" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13">
         <v>5</v>
       </c>
       <c r="D13" s="18">
@@ -15770,7 +15505,7 @@
       <c r="B14" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14">
         <v>50</v>
       </c>
       <c r="D14" s="18">
@@ -15789,7 +15524,7 @@
       <c r="B22" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22">
         <v>5</v>
       </c>
     </row>
@@ -15797,7 +15532,7 @@
       <c r="B23" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23">
         <v>9</v>
       </c>
     </row>
@@ -15805,7 +15540,7 @@
       <c r="B24" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24">
         <v>10</v>
       </c>
     </row>
@@ -15813,7 +15548,7 @@
       <c r="B25" s="15" t="s">
         <v>208</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25">
         <v>12</v>
       </c>
     </row>
@@ -15821,7 +15556,7 @@
       <c r="B26" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26">
         <v>14</v>
       </c>
     </row>
@@ -15829,7 +15564,7 @@
       <c r="B27" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="C27" s="22">
+      <c r="C27">
         <v>50</v>
       </c>
     </row>
@@ -15875,6 +15610,11 @@
       <c r="A41" s="19">
         <f>GETPIVOTDATA("Género",$B$34,"Género","Femenino")</f>
         <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EJERCICIOS DE NIVEL AVANZADO DE EXCEL
</commit_message>
<xml_diff>
--- a/Nivel Avanzado/Examen Nivel Avanzado.xlsx
+++ b/Nivel Avanzado/Examen Nivel Avanzado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\db\Nik Denilson\Cursos\EXCEL\Nivel Avanzado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A88E55-EB18-4F30-B853-05FCE0508CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F5F606-FE3D-4819-9F55-BA593D377982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="212">
   <si>
     <t>EXAMEN NIVEL AVANZADO- CCE</t>
   </si>
@@ -691,9 +691,6 @@
   </si>
   <si>
     <t>20-29</t>
-  </si>
-  <si>
-    <t>50-59</t>
   </si>
   <si>
     <t>30-39</t>
@@ -856,73 +853,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="46">
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
+  <dxfs count="32">
     <dxf>
       <font>
         <b/>
@@ -2809,7 +2740,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Administrativo</c:v>
+                  <c:v>Finanzas</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2821,7 +2752,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>4</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2917,7 +2848,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Administrativo</c:v>
+                  <c:v>Finanzas</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2929,7 +2860,7 @@
                 <c:formatCode>_-[$USD]\ * #,##0.00_-;\-[$USD]\ * #,##0.00_-;_-[$USD]\ * "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>320633.63</c:v>
+                  <c:v>181383.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3541,34 +3472,28 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>INFOME_EJER2!$B$22:$B$25</c:f>
+              <c:f>INFOME_EJER2!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>50-59</c:v>
+                  <c:v>30-39</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>20-29</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>30-39</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>INFOME_EJER2!$C$22:$C$25</c:f>
+              <c:f>INFOME_EJER2!$C$22:$C$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
                   <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
@@ -8980,6 +8905,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
+            <a:pPr marL="0" indent="0"/>
             <a:t>100.00%</a:t>
           </a:fld>
           <a:endParaRPr lang="es-PE" sz="3500" b="0" i="0" u="none" strike="noStrike" kern="1200">
@@ -10346,7 +10272,7 @@
     <dataField name="Suma de Venta" fld="8" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="34">
+    <format dxfId="20">
       <pivotArea dataOnly="0" fieldPosition="0">
         <references count="1">
           <reference field="4" count="0"/>
@@ -10515,14 +10441,14 @@
     <dataField name="Suma de Venta" fld="8" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="36">
+    <format dxfId="22">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
@@ -10562,8 +10488,8 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="8">
-        <item x="3"/>
-        <item h="1" x="1"/>
+        <item h="1" x="3"/>
+        <item x="1"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="5"/>
@@ -10613,10 +10539,10 @@
     <dataField name="Recuento" fld="8" subtotal="count" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="0">
+    <format dxfId="8">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -10634,15 +10560,15 @@
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{930B1D6C-C551-426D-A03D-5145DB90C3AB}" name="TablaDinámica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Edad">
-  <location ref="B21:C25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="B21:C24" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="8">
-        <item x="3"/>
-        <item h="1" x="1"/>
+        <item h="1" x="3"/>
+        <item x="1"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="5"/>
@@ -10686,15 +10612,12 @@
   <rowFields count="1">
     <field x="7"/>
   </rowFields>
-  <rowItems count="4">
+  <rowItems count="3">
     <i>
-      <x v="4"/>
+      <x v="2"/>
     </i>
     <i>
       <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
     </i>
     <i t="grand">
       <x/>
@@ -10707,10 +10630,10 @@
     <dataField name="Cantidad Empleados" fld="0" subtotal="count" baseField="7" baseItem="1"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="2">
+    <format dxfId="10">
       <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -10806,8 +10729,8 @@
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="8">
-        <item x="3"/>
-        <item h="1" x="1"/>
+        <item h="1" x="3"/>
+        <item x="1"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="5"/>
@@ -10853,7 +10776,7 @@
   </rowFields>
   <rowItems count="2">
     <i>
-      <x/>
+      <x v="1"/>
     </i>
     <i t="grand">
       <x/>
@@ -10875,10 +10798,10 @@
     <dataField name="Salario Anual" fld="4" baseField="3" baseItem="0" numFmtId="167"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="4">
+    <format dxfId="13">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -10888,7 +10811,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="11">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -10968,8 +10891,8 @@
   <data>
     <tabular pivotCacheId="1937416377">
       <items count="7">
-        <i x="3" s="1"/>
-        <i x="1"/>
+        <i x="3"/>
+        <i x="1" s="1"/>
         <i x="0"/>
         <i x="2"/>
         <i x="6"/>
@@ -11016,21 +10939,21 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC378051-9E72-4BB2-9AB0-F6E23C44A7CC}" name="ventas" displayName="ventas" ref="B18:J68" totalsRowShown="0">
   <autoFilter ref="B18:J68" xr:uid="{FC378051-9E72-4BB2-9AB0-F6E23C44A7CC}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{D476CF5C-0E1B-40EE-A62B-72E29404A39A}" name="Sale ID" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{CAEA63EE-5517-4029-80DE-DE7ABE2E5FE3}" name="Fecha_Venta" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{2C9B66F8-7131-4DF0-9EB5-8DA6CE795516}" name="AÑO" dataDxfId="43">
+    <tableColumn id="1" xr3:uid="{D476CF5C-0E1B-40EE-A62B-72E29404A39A}" name="Sale ID" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{CAEA63EE-5517-4029-80DE-DE7ABE2E5FE3}" name="Fecha_Venta" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{2C9B66F8-7131-4DF0-9EB5-8DA6CE795516}" name="AÑO" dataDxfId="29">
       <calculatedColumnFormula>YEAR(ventas[[#This Row],[Fecha_Venta]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{5CF4337F-83E1-4D83-A9C4-E333AA16FA95}" name="MES" dataDxfId="42">
+    <tableColumn id="10" xr3:uid="{5CF4337F-83E1-4D83-A9C4-E333AA16FA95}" name="MES" dataDxfId="28">
       <calculatedColumnFormula>MONTH(ventas[[#This Row],[Fecha_Venta]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{72DA8C50-CDA6-43E5-9431-CA09B2A1FCBE}" name="Categoria" dataDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{F2936085-E31D-4D2E-AEFB-560F58DED709}" name="Nombre Producto" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{52293038-8FA6-493E-80D2-45B3340AF0BE}" name="Unidades Vendidas" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{6EAB6895-F3DA-4781-8FF6-2EA5365F5DE0}" name="Precio" dataDxfId="38" dataCellStyle="Millares">
+    <tableColumn id="3" xr3:uid="{72DA8C50-CDA6-43E5-9431-CA09B2A1FCBE}" name="Categoria" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{F2936085-E31D-4D2E-AEFB-560F58DED709}" name="Nombre Producto" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{52293038-8FA6-493E-80D2-45B3340AF0BE}" name="Unidades Vendidas" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{6EAB6895-F3DA-4781-8FF6-2EA5365F5DE0}" name="Precio" dataDxfId="24" dataCellStyle="Millares">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ventas[[#This Row],[Nombre Producto]],precios[Nombre Producto],precios[Price (USD)],"-",0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{CD38CA07-791D-439F-AC3E-94E715454305}" name="Venta" dataDxfId="37">
+    <tableColumn id="8" xr3:uid="{CD38CA07-791D-439F-AC3E-94E715454305}" name="Venta" dataDxfId="23">
       <calculatedColumnFormula>PRODUCT(ventas[[#This Row],[Unidades Vendidas]:[Precio]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11051,7 +10974,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8E1BDC09-0A31-468E-854C-B0887DE35573}" name="RH" displayName="RH" ref="A23:I73" totalsRowShown="0" headerRowDxfId="33" headerRowBorderDxfId="32" tableBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8E1BDC09-0A31-468E-854C-B0887DE35573}" name="RH" displayName="RH" ref="A23:I73" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17">
   <autoFilter ref="A23:I73" xr:uid="{8E1BDC09-0A31-468E-854C-B0887DE35573}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{CA5BADCE-87A3-4C6C-8C9E-32804204CFD6}" name="Nombre"/>
@@ -11059,9 +10982,9 @@
     <tableColumn id="3" xr3:uid="{5A6F001D-C24B-403D-8DFA-ED4932F47AF0}" name="Apellido Materno"/>
     <tableColumn id="4" xr3:uid="{4C5A6D7B-ADA5-4DAD-8FCE-5614D22DCB1A}" name="Puesto"/>
     <tableColumn id="5" xr3:uid="{F917D2AA-F2F7-4449-8B16-DDBE5DBD687A}" name="Salario Anual (USD)"/>
-    <tableColumn id="6" xr3:uid="{5150356B-0BC9-4651-9491-E2CA4FBB946A}" name="Fecha Contratación" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{479B983A-A0DC-4CB3-83F9-1DA14406634A}" name="Fecha Nacimiento" dataDxfId="29"/>
-    <tableColumn id="9" xr3:uid="{40E590F7-C3A8-4023-B335-4C8D470BAB64}" name="EdadTrabajador" dataDxfId="28">
+    <tableColumn id="6" xr3:uid="{5150356B-0BC9-4651-9491-E2CA4FBB946A}" name="Fecha Contratación" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{479B983A-A0DC-4CB3-83F9-1DA14406634A}" name="Fecha Nacimiento" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{40E590F7-C3A8-4023-B335-4C8D470BAB64}" name="EdadTrabajador" dataDxfId="14">
       <calculatedColumnFormula>INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{B2B75107-054A-4454-B3A1-24B9FCDE6668}" name="Género"/>
@@ -14743,7 +14666,7 @@
       </c>
       <c r="H54" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I54" t="s">
         <v>13</v>
@@ -14833,7 +14756,7 @@
       </c>
       <c r="H57" s="5">
         <f ca="1">INT(YEARFRAC(RH[[#This Row],[Fecha Nacimiento]],TODAY(),1))</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I57" t="s">
         <v>13</v>
@@ -15357,13 +15280,13 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="8" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C7" s="22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" s="18">
-        <v>320633.63</v>
+        <v>181383.4</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -15371,10 +15294,10 @@
         <v>199</v>
       </c>
       <c r="C8" s="22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="18">
-        <v>320633.63</v>
+        <v>181383.4</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.3">
@@ -15398,23 +15321,15 @@
         <v>210</v>
       </c>
       <c r="C23" s="22">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" s="15" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="C24" s="22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B25" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="C25" s="22">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>